<commit_message>
Rename columns in final evaluation data for clarity and update output files
</commit_message>
<xml_diff>
--- a/Analyze-Report/final_model_evaluation.xlsx
+++ b/Analyze-Report/final_model_evaluation.xlsx
@@ -425,12 +425,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>ave_MAE</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>ave_SD</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -1010,7 +1010,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MAE(Accuracy)</t>
+          <t>ave_MAE (Accuracy)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1027,7 +1027,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Prediction Stability (SD)</t>
+          <t>ave_SD (Prediction Stability)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>

<commit_message>
Refactor final evaluation metrics: rename Adjusted Accuracy to Mean Adjusted MAE, update normalization calculations, and enhance column names for clarity in output files.
</commit_message>
<xml_diff>
--- a/Analyze-Report/final_model_evaluation.xlsx
+++ b/Analyze-Report/final_model_evaluation.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,62 +430,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ave_MAE</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ave_SD</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Avg_Time</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Avg_Cost</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Adjusted_Accuracy</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Norm_Adjusted_Accuracy</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Mean Adjusted MAE (kg CO₂e)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Norm. Mean Adjusted MAE</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Norm_Time</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Norm_Cost</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Efficiency</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Final_Score</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
@@ -974,17 +986,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>How it is Calculated</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>What it means</t>
         </is>
@@ -1044,17 +1056,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Adjusted Accuracy</t>
+          <t>Mean Adjusted MAE (kg CO₂e)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Adjusted Accuracy = MAE + (λ × SD); λ = 0.3</t>
+          <t>Mean Adjusted MAE = ave_MAE + (λ × ave_SD); λ = 0.3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Consider accuracy with variance (penalizes unstable models)</t>
+          <t>Mean absolute error penalized by prediction variance (lower is better)</t>
         </is>
       </c>
     </row>
@@ -1095,17 +1107,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Norm. Adjusted Accuracy</t>
+          <t>Norm. Mean Adjusted MAE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Best Adjusted Accuracy ÷ Model's Adjusted Accuracy (higher = better)</t>
+          <t>Best Mean Adjusted MAE ÷ Model's Mean Adjusted MAE (higher = better)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Normalized accuracy where higher is better (1 = best)</t>
+          <t>Normalized error metric where higher = better (1 = best)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor evaluation metrics: rename Mean Adjusted MAE to Adjusted MAE, update calculations for Adjusted MAE and RMSE, and enhance normalization metrics. Update output files to reflect new metric names and structures.
</commit_message>
<xml_diff>
--- a/Analyze-Report/final_model_evaluation.xlsx
+++ b/Analyze-Report/final_model_evaluation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/48675a5a4bf720b8/Documents/GitHub/NewToMe/Analyze-Report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="11_0B5D8FE73A141E098503DC74307FDA101AD8D259" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3AE5D0F-9C39-411E-9EBF-6A0521E36C32}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_0B5D8FE7EF14527E35A1C0743035329621302C65" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1457C8A5-7A4E-4A2B-806A-152199822E85}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-28650" yWindow="150" windowWidth="23010" windowHeight="13650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="evaluation" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="83">
   <si>
     <t>Model</t>
   </si>
@@ -35,10 +35,16 @@
     <t>ave_SD</t>
   </si>
   <si>
-    <t>Mean Adjusted MAE (kg CO₂e)</t>
-  </si>
-  <si>
-    <t>Norm. Mean Adjusted MAE</t>
+    <t>Adjusted MAE (kg CO₂e)</t>
+  </si>
+  <si>
+    <t>Norm. Adjusted MAE</t>
+  </si>
+  <si>
+    <t>Adjusted RMSE (kg CO₂e)</t>
+  </si>
+  <si>
+    <t>Norm. Adjusted RMSE</t>
   </si>
   <si>
     <t>Norm. RMSE</t>
@@ -155,12 +161,18 @@
     <t>Variation of model residuals around the truth (higher = less stable)</t>
   </si>
   <si>
-    <t>Mean Adjusted MAE = ave_MAE + (λ × ave_SD_resid); λ = 0.3</t>
+    <t>Adjusted MAE = MAE + (λ × SD_resid); λ = 0.3</t>
   </si>
   <si>
     <t>MAE penalized by residual variance (lower is better)</t>
   </si>
   <si>
+    <t>Adjusted RMSE = sqrt(RMSE**2 + (λ × SD_resid)**2); λ = 0.3</t>
+  </si>
+  <si>
+    <t>RMSE penalized by residual variance (lower is better)</t>
+  </si>
+  <si>
     <t>Avg Time (sec)(speed)</t>
   </si>
   <si>
@@ -179,40 +191,40 @@
     <t>Average cost in US dollars per prediction</t>
   </si>
   <si>
-    <t>Mean Adjusted MAE ÷ product true value (normalized per product) then averaged across products</t>
+    <t>Adjusted MAE ÷ product true value (normalized per product) then averaged across products</t>
   </si>
   <si>
     <t>Scale-invariant adjusted error used to compute S_adj (lower = better)</t>
   </si>
   <si>
-    <t>RMSE ÷ product true value (normalized per product) then averaged across products</t>
-  </si>
-  <si>
-    <t>Scale-invariant RMSE used to compute S_rmse (lower = better)</t>
+    <t>Adjusted RMSE ÷ product true value (normalized per product) then averaged across products</t>
+  </si>
+  <si>
+    <t>Scale-invariant adjusted RMSE used to compute S_rmse (lower = better)</t>
   </si>
   <si>
     <t>S_adj (error score from adjusted MAE)</t>
   </si>
   <si>
-    <t>best(ave_norm_mean_adjusted) ÷ model's ave_norm_mean_adjusted (higher = better)</t>
-  </si>
-  <si>
-    <t>Benefit-style score derived from normalized adjusted MAE (1 = best)</t>
-  </si>
-  <si>
-    <t>S_rmse (error score from RMSE)</t>
-  </si>
-  <si>
-    <t>best(ave_norm_RMSE) ÷ model's ave_norm_RMSE (higher = better)</t>
-  </si>
-  <si>
-    <t>Benefit-style score derived from normalized RMSE (1 = best)</t>
+    <t>best(ave_norm_Adjusted_MAE) ÷ model's ave_norm_Adjusted_MAE (higher = better)</t>
+  </si>
+  <si>
+    <t>Benefit-style score derived from normalized Adjusted MAE (1 = best)</t>
+  </si>
+  <si>
+    <t>S_rmse (error score from adjusted RMSE)</t>
+  </si>
+  <si>
+    <t>best(ave_norm_Adjusted_RMSE) ÷ model's ave_norm_Adjusted_RMSE (higher = better)</t>
+  </si>
+  <si>
+    <t>Benefit-style score derived from normalized Adjusted RMSE (1 = best)</t>
   </si>
   <si>
     <t>S_err (Combined error)</t>
   </si>
   <si>
-    <t>S_err = ALPHA × S_adj + (1-ALPHA) × S_rmse (ALPHA default 0.5)</t>
+    <t>S_err = ALPHA × S_adj + (1-ALPHA) × S_rmse (ALPHA default 0.6)</t>
   </si>
   <si>
     <t>Combined error score balancing typical and large-error sensitivity (higher = better)</t>
@@ -258,25 +270,14 @@
   </si>
   <si>
     <t>Final ranking of models (1 = best)</t>
-  </si>
-  <si>
-    <t>Brand</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -292,7 +293,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -300,31 +301,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -627,16 +609,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y34"/>
+  <dimension ref="A1:T13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.21875" customWidth="1"/>
-    <col min="5" max="5" width="21.5546875" customWidth="1"/>
-    <col min="19" max="19" width="27" customWidth="1"/>
-    <col min="24" max="24" width="27" customWidth="1"/>
+    <col min="1" max="1" width="30.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="5" max="5" width="25.6640625" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="19.88671875" customWidth="1"/>
+    <col min="9" max="9" width="22.109375" customWidth="1"/>
+    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -691,10 +677,16 @@
       <c r="R1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B2">
         <v>17.6402</v>
@@ -712,45 +704,51 @@
         <v>1.574876288899836</v>
       </c>
       <c r="G2">
+        <v>24.159332972366489</v>
+      </c>
+      <c r="H2">
+        <v>1.510655839458299</v>
+      </c>
+      <c r="I2">
         <v>1.5034784709241951</v>
       </c>
-      <c r="H2">
+      <c r="J2">
         <v>12.54156666666667</v>
       </c>
-      <c r="I2">
+      <c r="K2">
         <v>1.6186916666666669E-2</v>
       </c>
-      <c r="J2">
+      <c r="L2">
         <v>60</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
       </c>
       <c r="M2">
         <v>1</v>
       </c>
       <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2">
         <v>0.13343229314792149</v>
       </c>
-      <c r="O2">
+      <c r="Q2">
         <v>3.2590106266938423E-2</v>
       </c>
-      <c r="P2">
+      <c r="R2">
         <v>3.5811245568879011</v>
       </c>
-      <c r="Q2">
+      <c r="S2">
         <v>0.8216443492855352</v>
       </c>
-      <c r="R2">
+      <c r="T2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3">
         <v>26.408033333333339</v>
@@ -768,45 +766,51 @@
         <v>2.098220226184671</v>
       </c>
       <c r="G3">
+        <v>30.052667087760678</v>
+      </c>
+      <c r="H3">
+        <v>2.0242364862071098</v>
+      </c>
+      <c r="I3">
         <v>2.0164116330151249</v>
       </c>
-      <c r="H3">
+      <c r="J3">
         <v>1.994566666666667</v>
       </c>
-      <c r="I3">
+      <c r="K3">
         <v>5.2753333333333333E-4</v>
       </c>
-      <c r="J3">
+      <c r="L3">
         <v>60</v>
       </c>
-      <c r="K3">
+      <c r="M3">
         <v>0.75057721265216537</v>
       </c>
-      <c r="L3">
-        <v>0.74562080792814589</v>
-      </c>
-      <c r="M3">
-        <v>0.7485946507625576</v>
-      </c>
       <c r="N3">
+        <v>0.74628426557468441</v>
+      </c>
+      <c r="O3">
+        <v>0.74886003382117305</v>
+      </c>
+      <c r="P3">
         <v>0.83900429500150131</v>
       </c>
-      <c r="O3">
+      <c r="Q3">
         <v>1</v>
       </c>
-      <c r="P3">
+      <c r="R3">
         <v>2.7786543295231191E-2</v>
       </c>
-      <c r="Q3">
-        <v>0.77472636486027135</v>
-      </c>
-      <c r="R3">
+      <c r="S3">
+        <v>0.77493867130716365</v>
+      </c>
+      <c r="T3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4">
         <v>72.431366666666648</v>
@@ -824,45 +828,51 @@
         <v>2.6664893952870301</v>
       </c>
       <c r="G4">
+        <v>73.755149891392918</v>
+      </c>
+      <c r="H4">
+        <v>2.580085076687809</v>
+      </c>
+      <c r="I4">
         <v>2.5543224434499021</v>
       </c>
-      <c r="H4">
+      <c r="J4">
         <v>2.857766666666667</v>
       </c>
-      <c r="I4">
+      <c r="K4">
         <v>4.7775833333333316E-3</v>
       </c>
-      <c r="J4">
+      <c r="L4">
         <v>60</v>
       </c>
-      <c r="K4">
+      <c r="M4">
         <v>0.59061787070438387</v>
       </c>
-      <c r="L4">
-        <v>0.58860167586907652</v>
-      </c>
-      <c r="M4">
-        <v>0.58981139277026084</v>
-      </c>
       <c r="N4">
+        <v>0.58550621183314699</v>
+      </c>
+      <c r="O4">
+        <v>0.58857320715588912</v>
+      </c>
+      <c r="P4">
         <v>0.58557964844356825</v>
       </c>
-      <c r="O4">
+      <c r="Q4">
         <v>0.1104184474485877</v>
       </c>
-      <c r="P4">
+      <c r="R4">
         <v>0.98892126790928125</v>
       </c>
-      <c r="Q4">
-        <v>0.56520698385517332</v>
-      </c>
-      <c r="R4">
+      <c r="S4">
+        <v>0.56421643536367594</v>
+      </c>
+      <c r="T4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B5">
         <v>31.918537499999999</v>
@@ -880,45 +890,51 @@
         <v>2.466365258501316</v>
       </c>
       <c r="G5">
+        <v>34.605471169374589</v>
+      </c>
+      <c r="H5">
+        <v>2.3754221348735212</v>
+      </c>
+      <c r="I5">
         <v>2.3641763972273719</v>
       </c>
-      <c r="H5">
+      <c r="J5">
         <v>20.36311666666667</v>
       </c>
-      <c r="I5">
+      <c r="K5">
         <v>1.866625E-3</v>
       </c>
-      <c r="J5">
+      <c r="L5">
         <v>60</v>
       </c>
-      <c r="K5">
+      <c r="M5">
         <v>0.63854138533283156</v>
       </c>
-      <c r="L5">
-        <v>0.6359417481232742</v>
-      </c>
-      <c r="M5">
-        <v>0.63750153044900859</v>
-      </c>
       <c r="N5">
+        <v>0.63595258176673408</v>
+      </c>
+      <c r="O5">
+        <v>0.63750586390639263</v>
+      </c>
+      <c r="P5">
         <v>8.2180445527784377E-2</v>
       </c>
-      <c r="O5">
+      <c r="Q5">
         <v>0.28261345157742979</v>
       </c>
-      <c r="P5">
+      <c r="R5">
         <v>1.2132332704538771</v>
       </c>
-      <c r="Q5">
-        <v>0.536458963767246</v>
-      </c>
-      <c r="R5">
+      <c r="S5">
+        <v>0.53646243053315323</v>
+      </c>
+      <c r="T5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B6">
         <v>43.963866666666661</v>
@@ -936,45 +952,51 @@
         <v>2.541829965305745</v>
       </c>
       <c r="G6">
+        <v>49.014277101738507</v>
+      </c>
+      <c r="H6">
+        <v>2.449633647383969</v>
+      </c>
+      <c r="I6">
         <v>2.4249208255886598</v>
       </c>
-      <c r="H6">
+      <c r="J6">
         <v>35.279983333333327</v>
       </c>
-      <c r="I6">
+      <c r="K6">
         <v>2.2848833333333329E-3</v>
       </c>
-      <c r="J6">
+      <c r="L6">
         <v>60</v>
       </c>
-      <c r="K6">
+      <c r="M6">
         <v>0.61958365051801656</v>
       </c>
-      <c r="L6">
-        <v>0.6200113649317186</v>
-      </c>
-      <c r="M6">
-        <v>0.61975473628349742</v>
-      </c>
       <c r="N6">
+        <v>0.61668643434578596</v>
+      </c>
+      <c r="O6">
+        <v>0.61842476404912428</v>
+      </c>
+      <c r="P6">
         <v>4.7433412430777387E-2</v>
       </c>
-      <c r="O6">
+      <c r="Q6">
         <v>0.23087976808551289</v>
       </c>
-      <c r="P6">
+      <c r="R6">
         <v>3.543955689079695</v>
       </c>
-      <c r="Q6">
-        <v>0.51446278929569023</v>
-      </c>
-      <c r="R6">
+      <c r="S6">
+        <v>0.51339881150819167</v>
+      </c>
+      <c r="T6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B7">
         <v>73.135283333333334</v>
@@ -992,45 +1014,51 @@
         <v>5.135650873983181</v>
       </c>
       <c r="G7">
+        <v>81.714377671302017</v>
+      </c>
+      <c r="H7">
+        <v>4.9295614559960326</v>
+      </c>
+      <c r="I7">
         <v>4.8985295828500677</v>
       </c>
-      <c r="H7">
+      <c r="J7">
         <v>1.6734500000000001</v>
       </c>
-      <c r="I7">
+      <c r="K7">
         <v>5.4168666666666674E-4</v>
       </c>
-      <c r="J7">
+      <c r="L7">
         <v>60</v>
       </c>
-      <c r="K7">
+      <c r="M7">
         <v>0.30665563675263319</v>
       </c>
-      <c r="L7">
-        <v>0.30692444446770761</v>
-      </c>
-      <c r="M7">
-        <v>0.30676315983866298</v>
-      </c>
       <c r="N7">
+        <v>0.30644832262340871</v>
+      </c>
+      <c r="O7">
+        <v>0.30657271110094342</v>
+      </c>
+      <c r="P7">
         <v>1</v>
       </c>
-      <c r="O7">
+      <c r="Q7">
         <v>0.97387173401498073</v>
       </c>
-      <c r="P7">
+      <c r="R7">
         <v>6.6296077707471507E-2</v>
       </c>
-      <c r="Q7">
-        <v>0.44410411457167942</v>
-      </c>
-      <c r="R7">
+      <c r="S7">
+        <v>0.44395175558150368</v>
+      </c>
+      <c r="T7">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B8">
         <v>23.807199999999991</v>
@@ -1048,45 +1076,51 @@
         <v>3.636266911559682</v>
       </c>
       <c r="G8">
+        <v>24.40021209390823</v>
+      </c>
+      <c r="H8">
+        <v>3.5229421774358252</v>
+      </c>
+      <c r="I8">
         <v>3.517314380570447</v>
       </c>
-      <c r="H8">
+      <c r="J8">
         <v>6.0598000000000001</v>
       </c>
-      <c r="I8">
+      <c r="K8">
         <v>2.4276249999999999E-2</v>
       </c>
-      <c r="J8">
+      <c r="L8">
         <v>60</v>
       </c>
-      <c r="K8">
+      <c r="M8">
         <v>0.43310249968006359</v>
       </c>
-      <c r="L8">
-        <v>0.42745069341254899</v>
-      </c>
-      <c r="M8">
-        <v>0.43084177717305783</v>
-      </c>
       <c r="N8">
+        <v>0.42880517572343507</v>
+      </c>
+      <c r="O8">
+        <v>0.43138357009741218</v>
+      </c>
+      <c r="P8">
         <v>0.27615597874529257</v>
       </c>
-      <c r="O8">
+      <c r="Q8">
         <v>2.1730429300719958E-2</v>
       </c>
-      <c r="P8">
+      <c r="R8">
         <v>3.5022586164321998</v>
       </c>
-      <c r="Q8">
-        <v>0.38718334001527621</v>
-      </c>
-      <c r="R8">
+      <c r="S8">
+        <v>0.38761677435475972</v>
+      </c>
+      <c r="T8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B9">
         <v>21.626366666666669</v>
@@ -1104,45 +1138,51 @@
         <v>3.4146585828463438</v>
       </c>
       <c r="G9">
+        <v>30.42622122374064</v>
+      </c>
+      <c r="H9">
+        <v>3.2958798930534421</v>
+      </c>
+      <c r="I9">
         <v>3.2817778597970499</v>
       </c>
-      <c r="H9">
+      <c r="J9">
         <v>25.49785</v>
       </c>
-      <c r="I9">
+      <c r="K9">
         <v>1.9245399999999999E-2</v>
       </c>
-      <c r="J9">
+      <c r="L9">
         <v>60</v>
       </c>
-      <c r="K9">
+      <c r="M9">
         <v>0.46121046971191232</v>
       </c>
-      <c r="L9">
-        <v>0.45812926259966752</v>
-      </c>
-      <c r="M9">
-        <v>0.45997798686701441</v>
-      </c>
       <c r="N9">
+        <v>0.45834675063335067</v>
+      </c>
+      <c r="O9">
+        <v>0.46006498208048768</v>
+      </c>
+      <c r="P9">
         <v>6.5631023792238743E-2</v>
       </c>
-      <c r="O9">
+      <c r="Q9">
         <v>2.741087918702248E-2</v>
       </c>
-      <c r="P9">
+      <c r="R9">
         <v>10.612411117324349</v>
       </c>
-      <c r="Q9">
-        <v>0.3791975870217984</v>
-      </c>
-      <c r="R9">
+      <c r="S9">
+        <v>0.37926718319257707</v>
+      </c>
+      <c r="T9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B10">
         <v>35.946199999999997</v>
@@ -1160,45 +1200,51 @@
         <v>3.6314583963660092</v>
       </c>
       <c r="G10">
+        <v>38.983797287071852</v>
+      </c>
+      <c r="H10">
+        <v>3.5068076894962119</v>
+      </c>
+      <c r="I10">
         <v>3.4989210569821978</v>
       </c>
-      <c r="H10">
+      <c r="J10">
         <v>14.4358</v>
       </c>
-      <c r="I10">
+      <c r="K10">
         <v>1.8112699999999999E-2</v>
       </c>
-      <c r="J10">
+      <c r="L10">
         <v>60</v>
       </c>
-      <c r="K10">
+      <c r="M10">
         <v>0.43367598276118968</v>
       </c>
-      <c r="L10">
-        <v>0.42969774008605621</v>
-      </c>
-      <c r="M10">
-        <v>0.43208468569113628</v>
-      </c>
       <c r="N10">
+        <v>0.43077806746679309</v>
+      </c>
+      <c r="O10">
+        <v>0.43251681664343111</v>
+      </c>
+      <c r="P10">
         <v>0.1159236065892354</v>
       </c>
-      <c r="O10">
+      <c r="Q10">
         <v>2.912505227294707E-2</v>
       </c>
-      <c r="P10">
+      <c r="R10">
         <v>9.3989001710312898</v>
       </c>
-      <c r="Q10">
-        <v>0.36451254215494178</v>
-      </c>
-      <c r="R10">
+      <c r="S10">
+        <v>0.3648582469167776</v>
+      </c>
+      <c r="T10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B11">
         <v>42.844866666666661</v>
@@ -1216,45 +1262,51 @@
         <v>4.2417753159388862</v>
       </c>
       <c r="G11">
+        <v>48.613030671693927</v>
+      </c>
+      <c r="H11">
+        <v>4.1054109094008604</v>
+      </c>
+      <c r="I11">
         <v>4.0689194843978989</v>
       </c>
-      <c r="H11">
+      <c r="J11">
         <v>5.4298166666666674</v>
       </c>
-      <c r="I11">
+      <c r="K11">
         <v>1.09465E-2</v>
       </c>
-      <c r="J11">
+      <c r="L11">
         <v>60</v>
       </c>
-      <c r="K11">
+      <c r="M11">
         <v>0.3712776306144065</v>
       </c>
-      <c r="L11">
-        <v>0.3695031264909151</v>
-      </c>
-      <c r="M11">
-        <v>0.37056782896500989</v>
-      </c>
       <c r="N11">
+        <v>0.36796702517638957</v>
+      </c>
+      <c r="O11">
+        <v>0.36995338843919978</v>
+      </c>
+      <c r="P11">
         <v>0.3081964093325481</v>
       </c>
-      <c r="O11">
+      <c r="Q11">
         <v>4.8191964032808787E-2</v>
       </c>
-      <c r="P11">
+      <c r="R11">
         <v>2.5465912544312892</v>
       </c>
-      <c r="Q11">
-        <v>0.34509332277353061</v>
-      </c>
-      <c r="R11">
+      <c r="S11">
+        <v>0.34460177035288247</v>
+      </c>
+      <c r="T11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B12">
         <v>48.970866666666673</v>
@@ -1272,45 +1324,51 @@
         <v>4.7967876990288012</v>
       </c>
       <c r="G12">
+        <v>52.80590138883526</v>
+      </c>
+      <c r="H12">
+        <v>4.6131152165777527</v>
+      </c>
+      <c r="I12">
         <v>4.6013773475363369</v>
       </c>
-      <c r="H12">
+      <c r="J12">
         <v>5.8223333333333329</v>
       </c>
-      <c r="I12">
+      <c r="K12">
         <v>1.4697E-2</v>
       </c>
-      <c r="J12">
+      <c r="L12">
         <v>60</v>
       </c>
-      <c r="K12">
+      <c r="M12">
         <v>0.32831894753636298</v>
       </c>
-      <c r="L12">
-        <v>0.32674531066874118</v>
-      </c>
-      <c r="M12">
-        <v>0.32768949278931431</v>
-      </c>
       <c r="N12">
+        <v>0.32746978311537911</v>
+      </c>
+      <c r="O12">
+        <v>0.32797928176796942</v>
+      </c>
+      <c r="P12">
         <v>0.28741913322277091</v>
       </c>
-      <c r="O12">
+      <c r="Q12">
         <v>3.5893946676018189E-2</v>
       </c>
-      <c r="P12">
+      <c r="R12">
         <v>4.1904778533985994</v>
       </c>
-      <c r="Q12">
-        <v>0.30705916154866791</v>
-      </c>
-      <c r="R12">
+      <c r="S12">
+        <v>0.30729099273159199</v>
+      </c>
+      <c r="T12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B13">
         <v>97.669866666666664</v>
@@ -1328,207 +1386,67 @@
         <v>16.123911773815671</v>
       </c>
       <c r="G13">
+        <v>112.9899690239089</v>
+      </c>
+      <c r="H13">
+        <v>16.483249903105889</v>
+      </c>
+      <c r="I13">
         <v>16.215541562877029</v>
       </c>
-      <c r="H13">
+      <c r="J13">
         <v>6.9490666666666669</v>
       </c>
-      <c r="I13">
+      <c r="K13">
         <v>1.673761E-2</v>
       </c>
-      <c r="J13">
+      <c r="L13">
         <v>60</v>
       </c>
-      <c r="K13">
+      <c r="M13">
         <v>9.7673338268834384E-2</v>
       </c>
-      <c r="L13">
-        <v>9.2718363126834055E-2</v>
-      </c>
-      <c r="M13">
-        <v>9.5691348212034247E-2</v>
-      </c>
       <c r="N13">
+        <v>9.1647936440893196E-2</v>
+      </c>
+      <c r="O13">
+        <v>9.5263177537657895E-2</v>
+      </c>
+      <c r="P13">
         <v>0.24081651252936981</v>
       </c>
-      <c r="O13">
+      <c r="Q13">
         <v>3.1517841215192341E-2</v>
       </c>
-      <c r="P13">
+      <c r="R13">
         <v>11.36005717615185</v>
       </c>
-      <c r="Q13">
-        <v>0.11425144750979251</v>
-      </c>
-      <c r="R13">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="22" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S22" s="1"/>
-      <c r="T22" s="1"/>
-      <c r="W22" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="X22" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S23" s="1"/>
-      <c r="T23" s="1"/>
-      <c r="W23" s="2"/>
-      <c r="X23" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="Y23" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S24" s="1"/>
-      <c r="T24" s="1"/>
-      <c r="W24" s="2"/>
-      <c r="X24" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="Y24" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S25" s="1"/>
-      <c r="T25" s="1"/>
-      <c r="W25" s="2"/>
-      <c r="X25" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y25" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S26" s="1"/>
-      <c r="T26" s="1"/>
-      <c r="W26" s="2"/>
-      <c r="X26" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y26" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S27" s="1"/>
-      <c r="T27" s="1"/>
-      <c r="W27" s="2"/>
-      <c r="X27" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="Y27" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S28" s="1"/>
-      <c r="T28" s="1"/>
-      <c r="W28" s="2"/>
-      <c r="X28" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y28" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="29" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S29" s="1"/>
-      <c r="T29" s="1"/>
-      <c r="W29" s="2"/>
-      <c r="X29" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="Y29" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="30" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S30" s="1"/>
-      <c r="T30" s="1"/>
-      <c r="W30" s="2"/>
-      <c r="X30" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="Y30" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S31" s="1"/>
-      <c r="T31" s="1"/>
-      <c r="W31" s="2"/>
-      <c r="X31" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="Y31" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S32" s="1"/>
-      <c r="T32" s="1"/>
-      <c r="W32" s="2"/>
-      <c r="X32" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y32" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="33" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S33" s="1"/>
-      <c r="T33" s="1"/>
-      <c r="W33" s="2"/>
-      <c r="X33" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y33" s="1">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="34" spans="19:25" x14ac:dyDescent="0.3">
-      <c r="S34" s="1"/>
-      <c r="T34" s="1"/>
-      <c r="W34" s="2"/>
-      <c r="X34" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y34" s="1">
+      <c r="S13">
+        <v>0.1139089109702914</v>
+      </c>
+      <c r="T13">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -1536,43 +1454,43 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1580,142 +1498,153 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C18" t="s">
-        <v>78</v>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>